<commit_message>
update audit log week2
</commit_message>
<xml_diff>
--- a/Week1_AI_Audit_Log.xlsx
+++ b/Week1_AI_Audit_Log.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\FPT\SWP391\AI-Audit-Log\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AA3DCC92-2503-4122-A36A-073947000562}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFD872C5-BE55-407D-B9A7-86C297E1D3DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="16220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="16220" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1. Metadata &amp; Summary" sheetId="1" r:id="rId1"/>
@@ -644,14 +644,6 @@
     </font>
     <font>
       <b/>
-      <sz val="12"/>
-      <color theme="3" tint="0.39997558519241921"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -659,14 +651,6 @@
     </font>
     <font>
       <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
-      <color rgb="FF1F4E78"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -722,6 +706,21 @@
       <b/>
       <sz val="14"/>
       <color rgb="FF2E75B6"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="3" tint="0.39997558519241921"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="3" tint="0.39997558519241921"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -809,49 +808,47 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -860,6 +857,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1173,206 +1172,206 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-    </row>
-    <row r="3" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="2" t="s">
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+    </row>
+    <row r="3" spans="1:4" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A3" s="25" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="3" t="s">
         <v>183</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="3" t="s">
         <v>184</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="3" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A9" s="2" t="s">
+    <row r="9" spans="1:4" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A9" s="25" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="3" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="3" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="C12" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D12" s="4"/>
+      <c r="D12" s="3"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A15" s="5" t="s">
+    <row r="15" spans="1:4" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A15" s="25" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="9" t="s">
+      <c r="A16" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="B16" s="9" t="s">
+      <c r="B16" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="C16" s="9" t="s">
+      <c r="C16" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D16" s="9" t="s">
+      <c r="D16" s="7" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A17" s="6" t="s">
+      <c r="A17" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="B17" s="6" t="s">
+      <c r="B17" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="C17" s="6" t="s">
+      <c r="C17" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="D17" s="6" t="s">
+      <c r="D17" s="4" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A18" s="7" t="s">
+      <c r="A18" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="B18" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="C18" s="7" t="s">
+      <c r="C18" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="D18" s="7" t="s">
+      <c r="D18" s="5" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A19" s="6" t="s">
+      <c r="A19" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B19" s="6" t="s">
+      <c r="B19" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="C19" s="6" t="s">
+      <c r="C19" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="D19" s="6" t="s">
+      <c r="D19" s="4" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="22" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A22" s="5" t="s">
+    <row r="22" spans="1:4" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A22" s="25" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A23" s="9" t="s">
+      <c r="A23" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="B23" s="9" t="s">
+      <c r="B23" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="C23" s="9" t="s">
+      <c r="C23" s="7" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A24" s="6" t="s">
+      <c r="A24" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="B24" s="8">
+      <c r="B24" s="6">
         <v>3</v>
       </c>
-      <c r="C24" s="8" t="s">
+      <c r="C24" s="6" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A25" s="6" t="s">
+      <c r="A25" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="B25" s="8">
+      <c r="B25" s="6">
         <v>2</v>
       </c>
-      <c r="C25" s="8" t="s">
+      <c r="C25" s="6" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A26" s="6" t="s">
+      <c r="A26" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="B26" s="8">
+      <c r="B26" s="6">
         <v>3</v>
       </c>
-      <c r="C26" s="8" t="s">
+      <c r="C26" s="6" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A27" s="6" t="s">
+      <c r="A27" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="B27" s="8">
+      <c r="B27" s="6">
         <v>2</v>
       </c>
-      <c r="C27" s="8" t="s">
+      <c r="C27" s="6" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1400,312 +1399,312 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="21" x14ac:dyDescent="0.5">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10"/>
-      <c r="H1" s="10"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
+      <c r="H1" s="8"/>
     </row>
     <row r="2" spans="1:8" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="B2" s="18"/>
-      <c r="C2" s="18"/>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
-      <c r="F2" s="18"/>
-      <c r="G2" s="18"/>
-      <c r="H2" s="18"/>
+      <c r="B2" s="16"/>
+      <c r="C2" s="16"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="16"/>
+      <c r="G2" s="16"/>
+      <c r="H2" s="16"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A3" s="19" t="s">
+      <c r="A3" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="C3" s="19" t="s">
+      <c r="C3" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="D3" s="19" t="s">
+      <c r="D3" s="17" t="s">
         <v>42</v>
       </c>
-      <c r="E3" s="19" t="s">
+      <c r="E3" s="17" t="s">
         <v>43</v>
       </c>
-      <c r="F3" s="19" t="s">
+      <c r="F3" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="G3" s="19" t="s">
+      <c r="G3" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="H3" s="19" t="s">
+      <c r="H3" s="17" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="116" x14ac:dyDescent="0.35">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="B4" s="12" t="s">
+      <c r="B4" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="C4" s="12" t="s">
+      <c r="C4" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="D4" s="13" t="s">
+      <c r="D4" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="E4" s="13" t="s">
+      <c r="E4" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="F4" s="13" t="s">
+      <c r="F4" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="G4" s="13" t="s">
+      <c r="G4" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="H4" s="13" t="s">
+      <c r="H4" s="11" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="116" x14ac:dyDescent="0.35">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="C5" s="8" t="s">
+      <c r="C5" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="D5" s="14" t="s">
+      <c r="D5" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="E5" s="14" t="s">
+      <c r="E5" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="F5" s="14" t="s">
+      <c r="F5" s="12" t="s">
         <v>57</v>
       </c>
-      <c r="G5" s="14" t="s">
+      <c r="G5" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="H5" s="14" t="s">
+      <c r="H5" s="12" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="116" x14ac:dyDescent="0.35">
-      <c r="A6" s="12" t="s">
+      <c r="A6" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="B6" s="12" t="s">
+      <c r="B6" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="C6" s="12" t="s">
+      <c r="C6" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="D6" s="13" t="s">
+      <c r="D6" s="11" t="s">
         <v>62</v>
       </c>
-      <c r="E6" s="13" t="s">
+      <c r="E6" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="F6" s="13" t="s">
+      <c r="F6" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="G6" s="13" t="s">
+      <c r="G6" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="H6" s="13" t="s">
+      <c r="H6" s="11" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="101.5" x14ac:dyDescent="0.35">
-      <c r="A7" s="8" t="s">
+      <c r="A7" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="B7" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="C7" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="D7" s="14" t="s">
+      <c r="D7" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="E7" s="14" t="s">
+      <c r="E7" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="F7" s="14" t="s">
+      <c r="F7" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="G7" s="14" t="s">
+      <c r="G7" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="H7" s="14" t="s">
+      <c r="H7" s="12" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="101.5" x14ac:dyDescent="0.35">
-      <c r="A8" s="12" t="s">
+      <c r="A8" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="B8" s="12" t="s">
+      <c r="B8" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="C8" s="12" t="s">
+      <c r="C8" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="D8" s="13" t="s">
+      <c r="D8" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="E8" s="13" t="s">
+      <c r="E8" s="11" t="s">
         <v>75</v>
       </c>
-      <c r="F8" s="13" t="s">
+      <c r="F8" s="11" t="s">
         <v>76</v>
       </c>
-      <c r="G8" s="13" t="s">
+      <c r="G8" s="11" t="s">
         <v>77</v>
       </c>
-      <c r="H8" s="13" t="s">
+      <c r="H8" s="11" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="130.5" x14ac:dyDescent="0.35">
-      <c r="A9" s="8" t="s">
+      <c r="A9" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="B9" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="C9" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="D9" s="14" t="s">
+      <c r="D9" s="12" t="s">
         <v>80</v>
       </c>
-      <c r="E9" s="14" t="s">
+      <c r="E9" s="12" t="s">
         <v>81</v>
       </c>
-      <c r="F9" s="14" t="s">
+      <c r="F9" s="12" t="s">
         <v>82</v>
       </c>
-      <c r="G9" s="14" t="s">
+      <c r="G9" s="12" t="s">
         <v>83</v>
       </c>
-      <c r="H9" s="14" t="s">
+      <c r="H9" s="12" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="116" x14ac:dyDescent="0.35">
-      <c r="A10" s="12" t="s">
+      <c r="A10" s="10" t="s">
         <v>85</v>
       </c>
-      <c r="B10" s="12" t="s">
+      <c r="B10" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="C10" s="12" t="s">
+      <c r="C10" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="D10" s="13" t="s">
+      <c r="D10" s="11" t="s">
         <v>86</v>
       </c>
-      <c r="E10" s="13" t="s">
+      <c r="E10" s="11" t="s">
         <v>87</v>
       </c>
-      <c r="F10" s="13" t="s">
+      <c r="F10" s="11" t="s">
         <v>88</v>
       </c>
-      <c r="G10" s="13" t="s">
+      <c r="G10" s="11" t="s">
         <v>89</v>
       </c>
-      <c r="H10" s="13" t="s">
+      <c r="H10" s="11" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="101.5" x14ac:dyDescent="0.35">
-      <c r="A11" s="8" t="s">
+      <c r="A11" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="B11" s="8" t="s">
+      <c r="B11" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="C11" s="8" t="s">
+      <c r="C11" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="D11" s="14" t="s">
+      <c r="D11" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="E11" s="14" t="s">
+      <c r="E11" s="12" t="s">
         <v>93</v>
       </c>
-      <c r="F11" s="14" t="s">
+      <c r="F11" s="12" t="s">
         <v>94</v>
       </c>
-      <c r="G11" s="14" t="s">
+      <c r="G11" s="12" t="s">
         <v>95</v>
       </c>
-      <c r="H11" s="14" t="s">
+      <c r="H11" s="12" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="116" x14ac:dyDescent="0.35">
-      <c r="A12" s="12" t="s">
+      <c r="A12" s="10" t="s">
         <v>97</v>
       </c>
-      <c r="B12" s="12" t="s">
+      <c r="B12" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="C12" s="12" t="s">
+      <c r="C12" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="D12" s="13" t="s">
+      <c r="D12" s="11" t="s">
         <v>98</v>
       </c>
-      <c r="E12" s="13" t="s">
+      <c r="E12" s="11" t="s">
         <v>99</v>
       </c>
-      <c r="F12" s="13" t="s">
+      <c r="F12" s="11" t="s">
         <v>100</v>
       </c>
-      <c r="G12" s="13" t="s">
+      <c r="G12" s="11" t="s">
         <v>101</v>
       </c>
-      <c r="H12" s="13" t="s">
+      <c r="H12" s="11" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="116" x14ac:dyDescent="0.35">
-      <c r="A13" s="8" t="s">
+      <c r="A13" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="B13" s="8" t="s">
+      <c r="B13" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="C13" s="8" t="s">
+      <c r="C13" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="D13" s="14" t="s">
+      <c r="D13" s="12" t="s">
         <v>104</v>
       </c>
-      <c r="E13" s="14" t="s">
+      <c r="E13" s="12" t="s">
         <v>105</v>
       </c>
-      <c r="F13" s="14" t="s">
+      <c r="F13" s="12" t="s">
         <v>106</v>
       </c>
-      <c r="G13" s="14" t="s">
+      <c r="G13" s="12" t="s">
         <v>107</v>
       </c>
-      <c r="H13" s="14" t="s">
+      <c r="H13" s="12" t="s">
         <v>108</v>
       </c>
     </row>
@@ -1730,174 +1729,174 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="21" x14ac:dyDescent="0.5">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="13" t="s">
         <v>109</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
-      <c r="F1" s="15"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="15" t="s">
         <v>110</v>
       </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
+      <c r="B2" s="15"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A3" s="19" t="s">
+      <c r="A3" s="17" t="s">
         <v>111</v>
       </c>
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="17" t="s">
         <v>112</v>
       </c>
-      <c r="C3" s="19" t="s">
+      <c r="C3" s="17" t="s">
         <v>113</v>
       </c>
-      <c r="D3" s="19" t="s">
+      <c r="D3" s="17" t="s">
         <v>114</v>
       </c>
-      <c r="E3" s="19" t="s">
+      <c r="E3" s="17" t="s">
         <v>115</v>
       </c>
-      <c r="F3" s="19" t="s">
+      <c r="F3" s="17" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="B4" s="12" t="s">
+      <c r="B4" s="10" t="s">
         <v>117</v>
       </c>
-      <c r="C4" s="13" t="s">
+      <c r="C4" s="11" t="s">
         <v>118</v>
       </c>
-      <c r="D4" s="13" t="s">
+      <c r="D4" s="11" t="s">
         <v>119</v>
       </c>
-      <c r="E4" s="13" t="s">
+      <c r="E4" s="11" t="s">
         <v>120</v>
       </c>
-      <c r="F4" s="13" t="s">
+      <c r="F4" s="11" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="6" t="s">
         <v>122</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="C5" s="14" t="s">
+      <c r="C5" s="12" t="s">
         <v>124</v>
       </c>
-      <c r="D5" s="14" t="s">
+      <c r="D5" s="12" t="s">
         <v>125</v>
       </c>
-      <c r="E5" s="14" t="s">
+      <c r="E5" s="12" t="s">
         <v>126</v>
       </c>
-      <c r="F5" s="14" t="s">
+      <c r="F5" s="12" t="s">
         <v>127</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="A6" s="12" t="s">
+      <c r="A6" s="10" t="s">
         <v>97</v>
       </c>
-      <c r="B6" s="12" t="s">
+      <c r="B6" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="C6" s="13" t="s">
+      <c r="C6" s="11" t="s">
         <v>129</v>
       </c>
-      <c r="D6" s="13" t="s">
+      <c r="D6" s="11" t="s">
         <v>130</v>
       </c>
-      <c r="E6" s="13" t="s">
+      <c r="E6" s="11" t="s">
         <v>131</v>
       </c>
-      <c r="F6" s="13" t="s">
+      <c r="F6" s="11" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A9" s="2" t="s">
+    <row r="9" spans="1:6" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A9" s="25" t="s">
         <v>133</v>
       </c>
-      <c r="B9" s="20"/>
+      <c r="B9" s="18"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A10" s="19" t="s">
+      <c r="A10" s="17" t="s">
         <v>134</v>
       </c>
-      <c r="B10" s="19" t="s">
+      <c r="B10" s="17" t="s">
         <v>135</v>
       </c>
-      <c r="C10" s="19" t="s">
+      <c r="C10" s="17" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="29" x14ac:dyDescent="0.35">
-      <c r="A11" s="8" t="s">
+      <c r="A11" s="6" t="s">
         <v>117</v>
       </c>
-      <c r="B11" s="14" t="s">
+      <c r="B11" s="12" t="s">
         <v>137</v>
       </c>
-      <c r="C11" s="14" t="s">
+      <c r="C11" s="12" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="29" x14ac:dyDescent="0.35">
-      <c r="A12" s="8" t="s">
+      <c r="A12" s="6" t="s">
         <v>139</v>
       </c>
-      <c r="B12" s="14" t="s">
+      <c r="B12" s="12" t="s">
         <v>140</v>
       </c>
-      <c r="C12" s="14" t="s">
+      <c r="C12" s="12" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="29" x14ac:dyDescent="0.35">
-      <c r="A13" s="8" t="s">
+      <c r="A13" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="B13" s="14" t="s">
+      <c r="B13" s="12" t="s">
         <v>142</v>
       </c>
-      <c r="C13" s="14" t="s">
+      <c r="C13" s="12" t="s">
         <v>143</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="29" x14ac:dyDescent="0.35">
-      <c r="A14" s="8" t="s">
+      <c r="A14" s="6" t="s">
         <v>144</v>
       </c>
-      <c r="B14" s="14" t="s">
+      <c r="B14" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="C14" s="14" t="s">
+      <c r="C14" s="12" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="29" x14ac:dyDescent="0.35">
-      <c r="A15" s="8" t="s">
+      <c r="A15" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="B15" s="14" t="s">
+      <c r="B15" s="12" t="s">
         <v>147</v>
       </c>
-      <c r="C15" s="14" t="s">
+      <c r="C15" s="12" t="s">
         <v>148</v>
       </c>
     </row>
@@ -1923,255 +1922,255 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="21" x14ac:dyDescent="0.5">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="8" t="s">
         <v>149</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="14" t="s">
         <v>150</v>
       </c>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
-    </row>
-    <row r="4" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+    </row>
+    <row r="4" spans="1:4" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A4" s="25" t="s">
         <v>151</v>
       </c>
-      <c r="B4" s="20"/>
+      <c r="B4" s="26"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="17" t="s">
         <v>152</v>
       </c>
-      <c r="B5" s="19" t="s">
+      <c r="B5" s="17" t="s">
         <v>153</v>
       </c>
-      <c r="C5" s="19" t="s">
+      <c r="C5" s="17" t="s">
         <v>154</v>
       </c>
-      <c r="D5" s="19" t="s">
+      <c r="D5" s="17" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" s="8" t="s">
+      <c r="A6" s="6" t="s">
         <v>156</v>
       </c>
-      <c r="B6" s="14" t="s">
+      <c r="B6" s="12" t="s">
         <v>157</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="C6" s="6" t="s">
         <v>158</v>
       </c>
-      <c r="D6" s="14" t="s">
+      <c r="D6" s="12" t="s">
         <v>159</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A7" s="8" t="s">
+      <c r="A7" s="6" t="s">
         <v>160</v>
       </c>
-      <c r="B7" s="14" t="s">
+      <c r="B7" s="12" t="s">
         <v>161</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="C7" s="6" t="s">
         <v>158</v>
       </c>
-      <c r="D7" s="14"/>
+      <c r="D7" s="12"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A8" s="8" t="s">
+      <c r="A8" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="14" t="s">
+      <c r="B8" s="12" t="s">
         <v>162</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="C8" s="6" t="s">
         <v>158</v>
       </c>
-      <c r="D8" s="14"/>
+      <c r="D8" s="12"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A9" s="8" t="s">
+      <c r="A9" s="6" t="s">
         <v>163</v>
       </c>
-      <c r="B9" s="14" t="s">
+      <c r="B9" s="12" t="s">
         <v>164</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="C9" s="6" t="s">
         <v>158</v>
       </c>
-      <c r="D9" s="14"/>
+      <c r="D9" s="12"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" s="8" t="s">
+      <c r="A10" s="6" t="s">
         <v>165</v>
       </c>
-      <c r="B10" s="14" t="s">
+      <c r="B10" s="12" t="s">
         <v>166</v>
       </c>
-      <c r="C10" s="8" t="s">
+      <c r="C10" s="6" t="s">
         <v>158</v>
       </c>
-      <c r="D10" s="14"/>
-    </row>
-    <row r="12" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A12" s="2" t="s">
+      <c r="D10" s="12"/>
+    </row>
+    <row r="12" spans="1:4" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A12" s="25" t="s">
         <v>167</v>
       </c>
-      <c r="B12" s="20"/>
+      <c r="B12" s="18"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A13" s="19" t="s">
+      <c r="A13" s="17" t="s">
         <v>152</v>
       </c>
-      <c r="B13" s="19" t="s">
+      <c r="B13" s="17" t="s">
         <v>153</v>
       </c>
-      <c r="C13" s="19" t="s">
+      <c r="C13" s="17" t="s">
         <v>154</v>
       </c>
-      <c r="D13" s="19" t="s">
+      <c r="D13" s="17" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A14" s="8" t="s">
+      <c r="A14" s="6" t="s">
         <v>156</v>
       </c>
-      <c r="B14" s="14" t="s">
+      <c r="B14" s="12" t="s">
         <v>169</v>
       </c>
-      <c r="C14" s="8" t="s">
+      <c r="C14" s="6" t="s">
         <v>158</v>
       </c>
-      <c r="D14" s="8" t="s">
+      <c r="D14" s="6" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A15" s="8" t="s">
+      <c r="A15" s="6" t="s">
         <v>160</v>
       </c>
-      <c r="B15" s="14" t="s">
+      <c r="B15" s="12" t="s">
         <v>171</v>
       </c>
-      <c r="C15" s="8" t="s">
+      <c r="C15" s="6" t="s">
         <v>158</v>
       </c>
-      <c r="D15" s="8" t="s">
+      <c r="D15" s="6" t="s">
         <v>172</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A16" s="8" t="s">
+      <c r="A16" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B16" s="14" t="s">
+      <c r="B16" s="12" t="s">
         <v>173</v>
       </c>
-      <c r="C16" s="8" t="s">
+      <c r="C16" s="6" t="s">
         <v>158</v>
       </c>
-      <c r="D16" s="8" t="s">
+      <c r="D16" s="6" t="s">
         <v>174</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A17" s="8" t="s">
+      <c r="A17" s="6" t="s">
         <v>163</v>
       </c>
-      <c r="B17" s="14" t="s">
+      <c r="B17" s="12" t="s">
         <v>175</v>
       </c>
-      <c r="C17" s="8" t="s">
+      <c r="C17" s="6" t="s">
         <v>158</v>
       </c>
-      <c r="D17" s="8" t="s">
+      <c r="D17" s="6" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A18" s="8" t="s">
+      <c r="A18" s="6" t="s">
         <v>165</v>
       </c>
-      <c r="B18" s="14" t="s">
+      <c r="B18" s="12" t="s">
         <v>177</v>
       </c>
-      <c r="C18" s="8" t="s">
+      <c r="C18" s="6" t="s">
         <v>158</v>
       </c>
-      <c r="D18" s="8" t="s">
+      <c r="D18" s="6" t="s">
         <v>178</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A20" s="21" t="s">
+      <c r="A20" s="19" t="s">
         <v>179</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A21" s="3" t="s">
+      <c r="A21" s="2" t="s">
         <v>180</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A22" s="3" t="s">
+      <c r="A22" s="2" t="s">
         <v>181</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="A25" s="22" t="s">
+      <c r="A25" s="20" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A26" s="11" t="s">
+      <c r="A26" s="9" t="s">
         <v>185</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="29" x14ac:dyDescent="0.35">
-      <c r="A27" s="23" t="s">
+      <c r="A27" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="B27" s="24" t="s">
+      <c r="B27" s="22" t="s">
         <v>186</v>
       </c>
-      <c r="C27" s="24" t="s">
+      <c r="C27" s="22" t="s">
         <v>187</v>
       </c>
-      <c r="D27" s="24" t="s">
+      <c r="D27" s="22" t="s">
         <v>188</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A28" s="25" t="s">
+      <c r="A28" s="23" t="s">
         <v>47</v>
       </c>
-      <c r="B28" s="26"/>
-      <c r="C28" s="26"/>
-      <c r="D28" s="26"/>
+      <c r="B28" s="24"/>
+      <c r="C28" s="24"/>
+      <c r="D28" s="24"/>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A29" s="25" t="s">
+      <c r="A29" s="23" t="s">
         <v>54</v>
       </c>
-      <c r="B29" s="26"/>
-      <c r="C29" s="26"/>
-      <c r="D29" s="26"/>
+      <c r="B29" s="24"/>
+      <c r="C29" s="24"/>
+      <c r="D29" s="24"/>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A30" s="25" t="s">
+      <c r="A30" s="23" t="s">
         <v>60</v>
       </c>
-      <c r="B30" s="26"/>
-      <c r="C30" s="26"/>
-      <c r="D30" s="26"/>
+      <c r="B30" s="24"/>
+      <c r="C30" s="24"/>
+      <c r="D30" s="24"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>